<commit_message>
Add SMOTE, Reject Option Classification and LIME; re-run all experiments; product wording
- Group-balanced SMOTE (pre-processing) and Reject Option Classification (post-processing)
  added to the mitigation methods and FairCKD-Select candidates
- LIME explanations next to SHAP, plus a SHAP-vs-LIME agreement table in every report
- All 7 experiments, models, figures and PDF reports regenerated
- Removed Phase-II / thesis wording from app, reports, README and website

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xb1KJdmtBuFVZoAbKS8Q7n
</commit_message>
<xml_diff>
--- a/results/ALL_EXPERIMENTS_SUMMARY.xlsx
+++ b/results/ALL_EXPERIMENTS_SUMMARY.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
   <si>
     <t>Dataset</t>
   </si>
@@ -88,13 +88,7 @@
     <t>SVM</t>
   </si>
   <si>
-    <t>XGBoost + Unawareness</t>
-  </si>
-  <si>
-    <t>Logistic Regression + Unawareness</t>
-  </si>
-  <si>
-    <t>Logistic Regression + Exp. Gradient</t>
+    <t>XGBoost + Reject Option</t>
   </si>
   <si>
     <t>XGBoost + RW + TO (hybrid)</t>
@@ -106,16 +100,16 @@
     <t>XGBoost + Threshold Opt.</t>
   </si>
   <si>
-    <t>0.531 → 0.411</t>
-  </si>
-  <si>
-    <t>0.627 → 0.473</t>
-  </si>
-  <si>
-    <t>0.619 → 0.530</t>
-  </si>
-  <si>
-    <t>0.204 → 0.092</t>
+    <t>0.531 → 0.263</t>
+  </si>
+  <si>
+    <t>0.627 → 0.386</t>
+  </si>
+  <si>
+    <t>0.578 → 0.316</t>
+  </si>
+  <si>
+    <t>0.259 → 0.143</t>
   </si>
   <si>
     <t>0.069 → 0.012</t>
@@ -523,16 +517,16 @@
         <v>0.5639999999999999</v>
       </c>
       <c r="I2">
-        <v>0.392</v>
+        <v>0.305</v>
       </c>
       <c r="J2">
-        <v>0.721</v>
+        <v>0.71</v>
       </c>
       <c r="K2" t="s">
         <v>24</v>
       </c>
       <c r="L2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -561,16 +555,16 @@
         <v>0.6860000000000001</v>
       </c>
       <c r="I3">
-        <v>0.484</v>
+        <v>0.365</v>
       </c>
       <c r="J3">
-        <v>0.723</v>
+        <v>0.711</v>
       </c>
       <c r="K3" t="s">
         <v>24</v>
       </c>
       <c r="L3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -599,16 +593,16 @@
         <v>0.626</v>
       </c>
       <c r="I4">
-        <v>0.425</v>
+        <v>0.389</v>
       </c>
       <c r="J4">
-        <v>0.711</v>
+        <v>0.708</v>
       </c>
       <c r="K4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -637,16 +631,16 @@
         <v>0.259</v>
       </c>
       <c r="I5">
-        <v>0.128</v>
+        <v>0.113</v>
       </c>
       <c r="J5">
-        <v>0.719</v>
+        <v>0.721</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -675,16 +669,16 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="I6">
-        <v>0.031</v>
+        <v>0.028</v>
       </c>
       <c r="J6">
-        <v>0.727</v>
+        <v>0.726</v>
       </c>
       <c r="K6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -719,10 +713,10 @@
         <v>0.993</v>
       </c>
       <c r="K7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -751,16 +745,16 @@
         <v>0.138</v>
       </c>
       <c r="I8">
-        <v>0.043</v>
+        <v>0.039</v>
       </c>
       <c r="J8">
-        <v>0.908</v>
+        <v>0.909</v>
       </c>
       <c r="K8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>